<commit_message>
Added Unternehmens Beispiele and cleanup Nutzwerte
</commit_message>
<xml_diff>
--- a/Nutzwertanalyse.xlsx
+++ b/Nutzwertanalyse.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8a471988a8a86cc1/Studium/Bachelor/Artefakte/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="60" documentId="8_{07ADA279-FDEA-4443-8009-F886D968C4FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78058858-0CBA-4371-8DC0-8E39D3D9B04C}"/>
+  <xr:revisionPtr revIDLastSave="95" documentId="8_{07ADA279-FDEA-4443-8009-F886D968C4FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9EF3FEE-D319-4987-B75E-092467A297FF}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{20C679E4-C9D8-48C4-B659-4235CD5DE514}"/>
+    <workbookView xWindow="-28920" yWindow="345" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{20C679E4-C9D8-48C4-B659-4235CD5DE514}"/>
   </bookViews>
   <sheets>
     <sheet name="Szenarien" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="26">
   <si>
     <t>Szenario</t>
   </si>
@@ -101,13 +101,7 @@
     <t>Kriterium</t>
   </si>
   <si>
-    <t>Hochverfügbarkeit &amp; Ausfallsicherheit</t>
-  </si>
-  <si>
     <t>Hybrid-/Multi-Cloud-Fähigkeit</t>
-  </si>
-  <si>
-    <t>Usabiltiy in der Administration</t>
   </si>
   <si>
     <t>Gewichtung</t>
@@ -117,9 +111,6 @@
   </si>
   <si>
     <t>Nutzwert-Punkte</t>
-  </si>
-  <si>
-    <t>Vmware/Broadcom</t>
   </si>
   <si>
     <t>Nutanix</t>
@@ -150,6 +141,12 @@
   </si>
   <si>
     <t>#</t>
+  </si>
+  <si>
+    <t>Benutzerfreundlichkeit</t>
+  </si>
+  <si>
+    <t>VMware/Broadcom</t>
   </si>
 </sst>
 </file>
@@ -191,7 +188,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -255,11 +252,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -274,9 +295,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -286,11 +304,17 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -633,7 +657,7 @@
   <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:13" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -659,19 +683,19 @@
         <v>5</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="K1" s="7" t="s">
         <v>6</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -755,7 +779,7 @@
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="M3" s="12"/>
+      <c r="M3" s="13"/>
     </row>
     <row r="4" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7">
@@ -795,7 +819,7 @@
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="M4" s="12"/>
+      <c r="M4" s="13"/>
     </row>
     <row r="5" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7">
@@ -835,91 +859,91 @@
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="M5" s="12"/>
+      <c r="M5" s="13"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="9">
-        <v>5</v>
-      </c>
-      <c r="B6" s="10">
-        <v>5</v>
-      </c>
-      <c r="C6" s="10">
-        <v>15</v>
-      </c>
-      <c r="D6" s="10">
-        <v>10</v>
-      </c>
-      <c r="E6" s="10">
-        <v>10</v>
-      </c>
-      <c r="F6" s="10">
-        <v>15</v>
-      </c>
-      <c r="G6" s="10">
-        <v>15</v>
-      </c>
-      <c r="H6" s="10">
-        <v>10</v>
-      </c>
-      <c r="I6" s="10">
-        <v>5</v>
-      </c>
-      <c r="J6" s="10">
-        <v>5</v>
-      </c>
-      <c r="K6" s="10">
+      <c r="A6" s="8">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9">
+        <v>5</v>
+      </c>
+      <c r="C6" s="9">
+        <v>15</v>
+      </c>
+      <c r="D6" s="9">
+        <v>10</v>
+      </c>
+      <c r="E6" s="9">
+        <v>10</v>
+      </c>
+      <c r="F6" s="9">
+        <v>15</v>
+      </c>
+      <c r="G6" s="9">
+        <v>15</v>
+      </c>
+      <c r="H6" s="9">
+        <v>10</v>
+      </c>
+      <c r="I6" s="9">
+        <v>5</v>
+      </c>
+      <c r="J6" s="9">
+        <v>5</v>
+      </c>
+      <c r="K6" s="9">
         <v>10</v>
       </c>
       <c r="L6" s="4">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="M6" s="12"/>
+      <c r="M6" s="13"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="7">
         <v>0</v>
       </c>
-      <c r="B7" s="11">
-        <v>10</v>
-      </c>
-      <c r="C7" s="11">
-        <v>10</v>
-      </c>
-      <c r="D7" s="11">
-        <v>10</v>
-      </c>
-      <c r="E7" s="11">
-        <v>10</v>
-      </c>
-      <c r="F7" s="11">
-        <v>10</v>
-      </c>
-      <c r="G7" s="11">
-        <v>10</v>
-      </c>
-      <c r="H7" s="11">
-        <v>10</v>
-      </c>
-      <c r="I7" s="11">
-        <v>10</v>
-      </c>
-      <c r="J7" s="11">
-        <v>10</v>
-      </c>
-      <c r="K7" s="11">
+      <c r="B7" s="10">
+        <v>10</v>
+      </c>
+      <c r="C7" s="10">
+        <v>10</v>
+      </c>
+      <c r="D7" s="10">
+        <v>10</v>
+      </c>
+      <c r="E7" s="10">
+        <v>10</v>
+      </c>
+      <c r="F7" s="10">
+        <v>10</v>
+      </c>
+      <c r="G7" s="10">
+        <v>10</v>
+      </c>
+      <c r="H7" s="10">
+        <v>10</v>
+      </c>
+      <c r="I7" s="10">
+        <v>10</v>
+      </c>
+      <c r="J7" s="10">
+        <v>10</v>
+      </c>
+      <c r="K7" s="10">
         <v>10</v>
       </c>
       <c r="L7" s="4">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="M7" s="8"/>
+      <c r="M7" s="14"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B8" s="7">
         <f t="shared" ref="B8:K8" si="1">SUM(B2:B7)</f>
@@ -962,7 +986,7 @@
         <v>40</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="M8" s="4">
         <f>AVERAGE(B8:K8)</f>
@@ -971,7 +995,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="M2:M6"/>
+    <mergeCell ref="M2:M7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -982,7 +1006,7 @@
   <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19" bestFit="1" customWidth="1"/>
   </cols>
@@ -992,13 +1016,13 @@
         <v>9</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -1059,7 +1083,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B6" s="3">
         <v>3</v>
@@ -1073,7 +1097,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" s="3">
         <v>3</v>
@@ -1101,7 +1125,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B9" s="3">
         <v>2</v>
@@ -1115,7 +1139,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="B10" s="3">
         <v>3</v>
@@ -1143,7 +1167,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B12" s="6">
         <f>SUM(B2:B11)</f>
@@ -1174,7 +1198,7 @@
   <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.42578125" bestFit="1" customWidth="1"/>
@@ -1183,48 +1207,48 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="H1" s="13"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" s="11"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>15</v>
-      </c>
       <c r="E2" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1361,7 +1385,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B7" s="3" t="e" cm="1">
         <f t="array" ref="B7">INDEX(Szenarien!B:K, $B$1+1, 5)</f>
@@ -1394,7 +1418,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" s="3" t="e" cm="1">
         <f t="array" ref="B8">INDEX(Szenarien!B:K, $B$1+1, 6)</f>
@@ -1460,7 +1484,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B10" s="3" t="e" cm="1">
         <f t="array" ref="B10">INDEX(Szenarien!B:K, $B$1+1, 8)</f>
@@ -1493,7 +1517,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="B11" s="3" t="e" cm="1">
         <f t="array" ref="B11">INDEX(Szenarien!B:K, $B$1+1, 9)</f>
@@ -1559,7 +1583,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B13" s="6" t="e">
         <f>SUM(B3:B12)</f>
@@ -1583,7 +1607,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -1627,7 +1651,7 @@
   <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.42578125" bestFit="1" customWidth="1"/>
@@ -1636,48 +1660,48 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="5">
+        <v>1</v>
+      </c>
+      <c r="C1" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="5">
-        <v>1</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="H1" s="13"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" s="11"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>15</v>
-      </c>
       <c r="E2" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1814,7 +1838,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B7" s="3" cm="1">
         <f t="array" ref="B7">INDEX(Szenarien!B:K, $B$1+1, 5)</f>
@@ -1847,7 +1871,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" s="3" cm="1">
         <f t="array" ref="B8">INDEX(Szenarien!B:K, $B$1+1, 6)</f>
@@ -1913,7 +1937,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B10" s="3" cm="1">
         <f t="array" ref="B10">INDEX(Szenarien!B:K, $B$1+1, 8)</f>
@@ -1946,7 +1970,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="B11" s="3" cm="1">
         <f t="array" ref="B11">INDEX(Szenarien!B:K, $B$1+1, 9)</f>
@@ -2012,7 +2036,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B13" s="6">
         <f>SUM(B3:B12)</f>
@@ -2036,7 +2060,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -2080,7 +2104,7 @@
   <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.42578125" bestFit="1" customWidth="1"/>
@@ -2089,48 +2113,48 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="5">
+        <v>2</v>
+      </c>
+      <c r="C1" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="5">
-        <v>2</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="H1" s="13"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" s="11"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>15</v>
-      </c>
       <c r="E2" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -2267,7 +2291,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B7" s="3" cm="1">
         <f t="array" ref="B7">INDEX(Szenarien!B:K, $B$1+1, 5)</f>
@@ -2300,7 +2324,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" s="3" cm="1">
         <f t="array" ref="B8">INDEX(Szenarien!B:K, $B$1+1, 6)</f>
@@ -2366,7 +2390,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B10" s="3" cm="1">
         <f t="array" ref="B10">INDEX(Szenarien!B:K, $B$1+1, 8)</f>
@@ -2399,7 +2423,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="B11" s="3" cm="1">
         <f t="array" ref="B11">INDEX(Szenarien!B:K, $B$1+1, 9)</f>
@@ -2465,7 +2489,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B13" s="6">
         <f>SUM(B3:B12)</f>
@@ -2489,7 +2513,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -2533,7 +2557,7 @@
   <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.42578125" bestFit="1" customWidth="1"/>
@@ -2542,48 +2566,48 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="5">
+        <v>3</v>
+      </c>
+      <c r="C1" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="5">
-        <v>3</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="H1" s="13"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" s="11"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>15</v>
-      </c>
       <c r="E2" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -2720,7 +2744,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B7" s="3" cm="1">
         <f t="array" ref="B7">INDEX(Szenarien!B:K, $B$1+1, 5)</f>
@@ -2753,7 +2777,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" s="3" cm="1">
         <f t="array" ref="B8">INDEX(Szenarien!B:K, $B$1+1, 6)</f>
@@ -2819,7 +2843,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B10" s="3" cm="1">
         <f t="array" ref="B10">INDEX(Szenarien!B:K, $B$1+1, 8)</f>
@@ -2852,7 +2876,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="B11" s="3" cm="1">
         <f t="array" ref="B11">INDEX(Szenarien!B:K, $B$1+1, 9)</f>
@@ -2918,7 +2942,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B13" s="6">
         <f>SUM(B3:B12)</f>
@@ -2942,7 +2966,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -2986,7 +3010,7 @@
   <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.42578125" bestFit="1" customWidth="1"/>
@@ -2995,48 +3019,48 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B1" s="5">
         <v>4</v>
       </c>
-      <c r="C1" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="H1" s="13"/>
+      <c r="C1" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" s="11"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>15</v>
-      </c>
       <c r="E2" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -3173,7 +3197,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B7" s="3" cm="1">
         <f t="array" ref="B7">INDEX(Szenarien!B:K, $B$1+1, 5)</f>
@@ -3206,7 +3230,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" s="3" cm="1">
         <f t="array" ref="B8">INDEX(Szenarien!B:K, $B$1+1, 6)</f>
@@ -3272,7 +3296,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B10" s="3" cm="1">
         <f t="array" ref="B10">INDEX(Szenarien!B:K, $B$1+1, 8)</f>
@@ -3305,7 +3329,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="B11" s="3" cm="1">
         <f t="array" ref="B11">INDEX(Szenarien!B:K, $B$1+1, 9)</f>
@@ -3371,7 +3395,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B13" s="6">
         <f>SUM(B3:B12)</f>
@@ -3395,7 +3419,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -3439,7 +3463,7 @@
   <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.42578125" bestFit="1" customWidth="1"/>
@@ -3448,48 +3472,48 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="5">
+        <v>5</v>
+      </c>
+      <c r="C1" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="5">
-        <v>5</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="H1" s="13"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" s="11"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>15</v>
-      </c>
       <c r="E2" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -3626,7 +3650,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B7" s="3" cm="1">
         <f t="array" ref="B7">INDEX(Szenarien!B:K, $B$1+1, 5)</f>
@@ -3659,7 +3683,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" s="3" cm="1">
         <f t="array" ref="B8">INDEX(Szenarien!B:K, $B$1+1, 6)</f>
@@ -3725,7 +3749,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B10" s="3" cm="1">
         <f t="array" ref="B10">INDEX(Szenarien!B:K, $B$1+1, 8)</f>
@@ -3758,7 +3782,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="B11" s="3" cm="1">
         <f t="array" ref="B11">INDEX(Szenarien!B:K, $B$1+1, 9)</f>
@@ -3824,7 +3848,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B13" s="6">
         <f>SUM(B3:B12)</f>
@@ -3848,7 +3872,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -3892,7 +3916,7 @@
   <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.42578125" bestFit="1" customWidth="1"/>
@@ -3901,48 +3925,48 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B1" s="5">
         <v>6</v>
       </c>
-      <c r="C1" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="H1" s="13"/>
+      <c r="C1" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" s="11"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>15</v>
-      </c>
       <c r="E2" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -4079,7 +4103,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B7" s="3" cm="1">
         <f t="array" ref="B7">INDEX(Szenarien!B:K, $B$1+1, 5)</f>
@@ -4112,7 +4136,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" s="3" cm="1">
         <f t="array" ref="B8">INDEX(Szenarien!B:K, $B$1+1, 6)</f>
@@ -4178,7 +4202,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B10" s="3" cm="1">
         <f t="array" ref="B10">INDEX(Szenarien!B:K, $B$1+1, 8)</f>
@@ -4211,7 +4235,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="B11" s="3" cm="1">
         <f t="array" ref="B11">INDEX(Szenarien!B:K, $B$1+1, 9)</f>
@@ -4277,7 +4301,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B13" s="6">
         <f>SUM(B3:B12)</f>
@@ -4301,7 +4325,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>

</xml_diff>

<commit_message>
Added normalization for values
</commit_message>
<xml_diff>
--- a/Nutzwertanalyse.xlsx
+++ b/Nutzwertanalyse.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8a471988a8a86cc1/Studium/Bachelor/Artefakte/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="95" documentId="8_{07ADA279-FDEA-4443-8009-F886D968C4FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9EF3FEE-D319-4987-B75E-092467A297FF}"/>
+  <xr:revisionPtr revIDLastSave="111" documentId="8_{07ADA279-FDEA-4443-8009-F886D968C4FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A15149CF-E0A2-4971-BFC3-A763001819A3}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="345" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{20C679E4-C9D8-48C4-B659-4235CD5DE514}"/>
+    <workbookView xWindow="-28920" yWindow="345" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{20C679E4-C9D8-48C4-B659-4235CD5DE514}"/>
   </bookViews>
   <sheets>
     <sheet name="Szenarien" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="27">
   <si>
     <t>Szenario</t>
   </si>
@@ -147,6 +147,9 @@
   </si>
   <si>
     <t>VMware/Broadcom</t>
+  </si>
+  <si>
+    <t>Normiert</t>
   </si>
 </sst>
 </file>
@@ -1195,7 +1198,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AE1F278-3573-456D-9F04-D37AF5426834}">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
@@ -1607,34 +1610,55 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
       <c r="D14" s="6" t="e">
-        <f>1+(F13&gt;D13)+(H13&gt;D13)</f>
+        <f>(D13-100)/2</f>
         <v>#VALUE!</v>
       </c>
       <c r="E14" s="6"/>
       <c r="F14" s="6" t="e">
-        <f>1+(D13&gt;F13)+(H13&gt;F13)</f>
+        <f>(F13-100)/2</f>
         <v>#VALUE!</v>
       </c>
       <c r="G14" s="6"/>
       <c r="H14" s="6" t="e">
+        <f>(H13-100)/2</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6" t="e">
+        <f>1+(F13&gt;D13)+(H13&gt;D13)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6" t="e">
+        <f>1+(D13&gt;F13)+(H13&gt;F13)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6" t="e">
         <f>1+(D13&gt;H13)+(F13&gt;H13)</f>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1648,7 +1672,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{221A8880-D037-4F7B-AF8F-E0B2DBB4D0DD}">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
@@ -2060,34 +2084,55 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
       <c r="D14" s="6">
-        <f>1+(F13&gt;D13)+(H13&gt;D13)</f>
-        <v>3</v>
+        <f>(D13-100)/2</f>
+        <v>47.5</v>
       </c>
       <c r="E14" s="6"/>
       <c r="F14" s="6">
-        <f>1+(D13&gt;F13)+(H13&gt;F13)</f>
-        <v>2</v>
+        <f>(F13-100)/2</f>
+        <v>55</v>
       </c>
       <c r="G14" s="6"/>
       <c r="H14" s="6">
+        <f>(H13-100)/2</f>
+        <v>77.5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6">
+        <f>1+(F13&gt;D13)+(H13&gt;D13)</f>
+        <v>3</v>
+      </c>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6">
+        <f>1+(D13&gt;F13)+(H13&gt;F13)</f>
+        <v>2</v>
+      </c>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6">
         <f>1+(D13&gt;H13)+(F13&gt;H13)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2101,7 +2146,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F5D9049-AE8F-48E7-96CF-575B5EEDD492}">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
@@ -2513,34 +2558,55 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
       <c r="D14" s="6">
-        <f>1+(F13&gt;D13)+(H13&gt;D13)</f>
-        <v>1</v>
+        <f>(D13-100)/2</f>
+        <v>67.5</v>
       </c>
       <c r="E14" s="6"/>
       <c r="F14" s="6">
-        <f>1+(D13&gt;F13)+(H13&gt;F13)</f>
-        <v>2</v>
+        <f>(F13-100)/2</f>
+        <v>57.5</v>
       </c>
       <c r="G14" s="6"/>
       <c r="H14" s="6">
+        <f>(H13-100)/2</f>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6">
+        <f>1+(F13&gt;D13)+(H13&gt;D13)</f>
+        <v>1</v>
+      </c>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6">
+        <f>1+(D13&gt;F13)+(H13&gt;F13)</f>
+        <v>2</v>
+      </c>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6">
         <f>1+(D13&gt;H13)+(F13&gt;H13)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2554,7 +2620,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4C83448-F0BC-46FC-BBB4-E081BD91570E}">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
@@ -2966,34 +3032,55 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
       <c r="D14" s="6">
-        <f>1+(F13&gt;D13)+(H13&gt;D13)</f>
-        <v>2</v>
+        <f>(D13-100)/2</f>
+        <v>55</v>
       </c>
       <c r="E14" s="6"/>
       <c r="F14" s="6">
-        <f>1+(D13&gt;F13)+(H13&gt;F13)</f>
-        <v>1</v>
+        <f>(F13-100)/2</f>
+        <v>70</v>
       </c>
       <c r="G14" s="6"/>
       <c r="H14" s="6">
+        <f>(H13-100)/2</f>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6">
+        <f>1+(F13&gt;D13)+(H13&gt;D13)</f>
+        <v>2</v>
+      </c>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6">
+        <f>1+(D13&gt;F13)+(H13&gt;F13)</f>
+        <v>1</v>
+      </c>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6">
         <f>1+(D13&gt;H13)+(F13&gt;H13)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3007,7 +3094,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{920EB601-A1EC-4140-BB2C-E4DAC592EC40}">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
@@ -3419,34 +3506,55 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
       <c r="D14" s="6">
-        <f>1+(F13&gt;D13)+(H13&gt;D13)</f>
-        <v>2</v>
+        <f>(D13-100)/2</f>
+        <v>65</v>
       </c>
       <c r="E14" s="6"/>
       <c r="F14" s="6">
-        <f>1+(D13&gt;F13)+(H13&gt;F13)</f>
-        <v>1</v>
+        <f>(F13-100)/2</f>
+        <v>72.5</v>
       </c>
       <c r="G14" s="6"/>
       <c r="H14" s="6">
+        <f>(H13-100)/2</f>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6">
+        <f>1+(F13&gt;D13)+(H13&gt;D13)</f>
+        <v>2</v>
+      </c>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6">
+        <f>1+(D13&gt;F13)+(H13&gt;F13)</f>
+        <v>1</v>
+      </c>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6">
         <f>1+(D13&gt;H13)+(F13&gt;H13)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3460,7 +3568,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0383F71C-DFA9-4483-8482-DC0F39D93A94}">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
@@ -3872,34 +3980,55 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
       <c r="D14" s="6">
-        <f>1+(F13&gt;D13)+(H13&gt;D13)</f>
-        <v>1</v>
+        <f>(D13-100)/2</f>
+        <v>77.5</v>
       </c>
       <c r="E14" s="6"/>
       <c r="F14" s="6">
-        <f>1+(D13&gt;F13)+(H13&gt;F13)</f>
-        <v>2</v>
+        <f>(F13-100)/2</f>
+        <v>67.5</v>
       </c>
       <c r="G14" s="6"/>
       <c r="H14" s="6">
+        <f>(H13-100)/2</f>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6">
+        <f>1+(F13&gt;D13)+(H13&gt;D13)</f>
+        <v>1</v>
+      </c>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6">
+        <f>1+(D13&gt;F13)+(H13&gt;F13)</f>
+        <v>2</v>
+      </c>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6">
         <f>1+(D13&gt;H13)+(F13&gt;H13)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3913,7 +4042,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65EF8FD4-0E48-4BC3-A71A-44B08418BCE9}">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
@@ -4325,34 +4454,55 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
       <c r="D14" s="6">
-        <f>1+(F13&gt;D13)+(H13&gt;D13)</f>
-        <v>1</v>
+        <f>(D13-100)/2</f>
+        <v>70</v>
       </c>
       <c r="E14" s="6"/>
       <c r="F14" s="6">
-        <f>1+(D13&gt;F13)+(H13&gt;F13)</f>
-        <v>2</v>
+        <f>(F13-100)/2</f>
+        <v>65</v>
       </c>
       <c r="G14" s="6"/>
       <c r="H14" s="6">
+        <f>(H13-100)/2</f>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6">
+        <f>1+(F13&gt;D13)+(H13&gt;D13)</f>
+        <v>1</v>
+      </c>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6">
+        <f>1+(D13&gt;F13)+(H13&gt;F13)</f>
+        <v>2</v>
+      </c>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6">
         <f>1+(D13&gt;H13)+(F13&gt;H13)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Fix: Woring for Nutzwerte, Punkte, Score...
</commit_message>
<xml_diff>
--- a/Nutzwertanalyse.xlsx
+++ b/Nutzwertanalyse.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8a471988a8a86cc1/Studium/Bachelor/Artefakte/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="111" documentId="8_{07ADA279-FDEA-4443-8009-F886D968C4FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A15149CF-E0A2-4971-BFC3-A763001819A3}"/>
+  <xr:revisionPtr revIDLastSave="137" documentId="8_{07ADA279-FDEA-4443-8009-F886D968C4FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4B3975B-ED8F-4DA6-83CD-481E9B57CD2C}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="345" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{20C679E4-C9D8-48C4-B659-4235CD5DE514}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{20C679E4-C9D8-48C4-B659-4235CD5DE514}"/>
   </bookViews>
   <sheets>
     <sheet name="Szenarien" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
     <sheet name="Szenario 3" sheetId="11" r:id="rId6"/>
     <sheet name="Szenario 4" sheetId="12" r:id="rId7"/>
     <sheet name="Szenario 5" sheetId="13" r:id="rId8"/>
-    <sheet name="Szenario 0 - Neutral" sheetId="15" r:id="rId9"/>
+    <sheet name="Szenario 0 - Referenz" sheetId="15" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="25">
   <si>
     <t>Szenario</t>
   </si>
@@ -107,12 +107,6 @@
     <t>Gewichtung</t>
   </si>
   <si>
-    <t>Punkte</t>
-  </si>
-  <si>
-    <t>Nutzwert-Punkte</t>
-  </si>
-  <si>
     <t>Nutanix</t>
   </si>
   <si>
@@ -120,12 +114,6 @@
   </si>
   <si>
     <t>Rang</t>
-  </si>
-  <si>
-    <t>SUMME</t>
-  </si>
-  <si>
-    <t>Mittelwert:</t>
   </si>
   <si>
     <t>Unified Storage</t>
@@ -149,7 +137,13 @@
     <t>VMware/Broadcom</t>
   </si>
   <si>
-    <t>Normiert</t>
+    <t>Score</t>
+  </si>
+  <si>
+    <t>Bewertung</t>
+  </si>
+  <si>
+    <t>Normiert (0-100)</t>
   </si>
 </sst>
 </file>
@@ -657,7 +651,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B54B5B26-C307-4627-BFB9-E5F80460B961}">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:13" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -686,19 +680,19 @@
         <v>5</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="K1" s="7" t="s">
         <v>6</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -943,58 +937,6 @@
         <v>100</v>
       </c>
       <c r="M7" s="14"/>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="7">
-        <f t="shared" ref="B8:K8" si="1">SUM(B2:B7)</f>
-        <v>105</v>
-      </c>
-      <c r="C8" s="7">
-        <f t="shared" si="1"/>
-        <v>60</v>
-      </c>
-      <c r="D8" s="7">
-        <f t="shared" si="1"/>
-        <v>60</v>
-      </c>
-      <c r="E8" s="7">
-        <f t="shared" si="1"/>
-        <v>55</v>
-      </c>
-      <c r="F8" s="7">
-        <f t="shared" si="1"/>
-        <v>70</v>
-      </c>
-      <c r="G8" s="7">
-        <f t="shared" si="1"/>
-        <v>40</v>
-      </c>
-      <c r="H8" s="7">
-        <f t="shared" si="1"/>
-        <v>60</v>
-      </c>
-      <c r="I8" s="7">
-        <f t="shared" si="1"/>
-        <v>45</v>
-      </c>
-      <c r="J8" s="7">
-        <f t="shared" si="1"/>
-        <v>65</v>
-      </c>
-      <c r="K8" s="7">
-        <f t="shared" si="1"/>
-        <v>40</v>
-      </c>
-      <c r="L8" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="M8" s="4">
-        <f>AVERAGE(B8:K8)</f>
-        <v>60</v>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1006,7 +948,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1C0522C-D307-4272-8586-B326A6E69815}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
@@ -1019,13 +961,13 @@
         <v>9</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -1128,7 +1070,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B9" s="3">
         <v>2</v>
@@ -1142,7 +1084,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B10" s="3">
         <v>3</v>
@@ -1169,27 +1111,10 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12" s="6">
-        <f>SUM(B2:B11)</f>
-        <v>24</v>
-      </c>
-      <c r="C12" s="6">
-        <f t="shared" ref="C12:D12" si="0">SUM(C2:C11)</f>
-        <v>23</v>
-      </c>
-      <c r="D12" s="6">
-        <f t="shared" si="0"/>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -1210,21 +1135,21 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D1" s="11"/>
       <c r="E1" s="11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F1" s="11"/>
       <c r="G1" s="11" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="H1" s="11"/>
     </row>
@@ -1236,22 +1161,22 @@
         <v>11</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1487,7 +1412,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B10" s="3" t="e" cm="1">
         <f t="array" ref="B10">INDEX(Szenarien!B:K, $B$1+1, 8)</f>
@@ -1520,7 +1445,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B11" s="3" t="e" cm="1">
         <f t="array" ref="B11">INDEX(Szenarien!B:K, $B$1+1, 9)</f>
@@ -1586,7 +1511,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B13" s="6" t="e">
         <f>SUM(B3:B12)</f>
@@ -1610,7 +1535,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -1631,7 +1556,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -1684,21 +1609,21 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B1" s="5">
         <v>1</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D1" s="11"/>
       <c r="E1" s="11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F1" s="11"/>
       <c r="G1" s="11" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="H1" s="11"/>
     </row>
@@ -1710,22 +1635,22 @@
         <v>11</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1961,7 +1886,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B10" s="3" cm="1">
         <f t="array" ref="B10">INDEX(Szenarien!B:K, $B$1+1, 8)</f>
@@ -1994,7 +1919,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B11" s="3" cm="1">
         <f t="array" ref="B11">INDEX(Szenarien!B:K, $B$1+1, 9)</f>
@@ -2060,7 +1985,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B13" s="6">
         <f>SUM(B3:B12)</f>
@@ -2084,7 +2009,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -2105,7 +2030,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -2158,21 +2083,21 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B1" s="5">
         <v>2</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D1" s="11"/>
       <c r="E1" s="11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F1" s="11"/>
       <c r="G1" s="11" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="H1" s="11"/>
     </row>
@@ -2184,22 +2109,22 @@
         <v>11</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -2435,7 +2360,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B10" s="3" cm="1">
         <f t="array" ref="B10">INDEX(Szenarien!B:K, $B$1+1, 8)</f>
@@ -2468,7 +2393,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B11" s="3" cm="1">
         <f t="array" ref="B11">INDEX(Szenarien!B:K, $B$1+1, 9)</f>
@@ -2534,7 +2459,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B13" s="6">
         <f>SUM(B3:B12)</f>
@@ -2558,7 +2483,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -2579,7 +2504,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -2632,21 +2557,21 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B1" s="5">
         <v>3</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D1" s="11"/>
       <c r="E1" s="11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F1" s="11"/>
       <c r="G1" s="11" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="H1" s="11"/>
     </row>
@@ -2658,22 +2583,22 @@
         <v>11</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -2909,7 +2834,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B10" s="3" cm="1">
         <f t="array" ref="B10">INDEX(Szenarien!B:K, $B$1+1, 8)</f>
@@ -2942,7 +2867,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B11" s="3" cm="1">
         <f t="array" ref="B11">INDEX(Szenarien!B:K, $B$1+1, 9)</f>
@@ -3008,7 +2933,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B13" s="6">
         <f>SUM(B3:B12)</f>
@@ -3032,7 +2957,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -3053,7 +2978,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -3106,21 +3031,21 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B1" s="5">
         <v>4</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D1" s="11"/>
       <c r="E1" s="11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F1" s="11"/>
       <c r="G1" s="11" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="H1" s="11"/>
     </row>
@@ -3132,22 +3057,22 @@
         <v>11</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -3383,7 +3308,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B10" s="3" cm="1">
         <f t="array" ref="B10">INDEX(Szenarien!B:K, $B$1+1, 8)</f>
@@ -3416,7 +3341,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B11" s="3" cm="1">
         <f t="array" ref="B11">INDEX(Szenarien!B:K, $B$1+1, 9)</f>
@@ -3482,7 +3407,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B13" s="6">
         <f>SUM(B3:B12)</f>
@@ -3506,7 +3431,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -3527,7 +3452,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -3580,21 +3505,21 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B1" s="5">
         <v>5</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D1" s="11"/>
       <c r="E1" s="11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F1" s="11"/>
       <c r="G1" s="11" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="H1" s="11"/>
     </row>
@@ -3606,22 +3531,22 @@
         <v>11</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -3857,7 +3782,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B10" s="3" cm="1">
         <f t="array" ref="B10">INDEX(Szenarien!B:K, $B$1+1, 8)</f>
@@ -3890,7 +3815,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B11" s="3" cm="1">
         <f t="array" ref="B11">INDEX(Szenarien!B:K, $B$1+1, 9)</f>
@@ -3956,7 +3881,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B13" s="6">
         <f>SUM(B3:B12)</f>
@@ -3980,7 +3905,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -4001,7 +3926,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -4054,21 +3979,21 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B1" s="5">
         <v>6</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D1" s="11"/>
       <c r="E1" s="11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F1" s="11"/>
       <c r="G1" s="11" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="H1" s="11"/>
     </row>
@@ -4080,22 +4005,22 @@
         <v>11</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -4331,7 +4256,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B10" s="3" cm="1">
         <f t="array" ref="B10">INDEX(Szenarien!B:K, $B$1+1, 8)</f>
@@ -4364,7 +4289,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B11" s="3" cm="1">
         <f t="array" ref="B11">INDEX(Szenarien!B:K, $B$1+1, 9)</f>
@@ -4430,7 +4355,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B13" s="6">
         <f>SUM(B3:B12)</f>
@@ -4454,7 +4379,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -4475,7 +4400,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>

</xml_diff>